<commit_message>
Week 4: Final Features Complete
</commit_message>
<xml_diff>
--- a/Data/TeamTracker.xlsx
+++ b/Data/TeamTracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\HROnboardingApp\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{290A2C58-7E48-4AB1-B0EB-949A51E4EB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B2DB88E-8BC7-43B1-9BFA-034378D0886F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{30C4A489-88FD-4F42-90A7-1AA7E270F543}"/>
   </bookViews>
@@ -173,7 +173,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="801">
   <si>
     <t>SrNo</t>
   </si>
@@ -1503,6 +1503,9 @@
     <t>Senior Consultant</t>
   </si>
   <si>
+    <t>2026-08-01</t>
+  </si>
+  <si>
     <t>AWS</t>
   </si>
   <si>
@@ -1515,6 +1518,36 @@
     <t>7937937830</t>
   </si>
   <si>
+    <t>Rahul Patki</t>
+  </si>
+  <si>
+    <t>rpatki@deloitte.com</t>
+  </si>
+  <si>
+    <t>2026-09-07</t>
+  </si>
+  <si>
+    <t>Firewire Rsik</t>
+  </si>
+  <si>
+    <t>Working on VDI setup</t>
+  </si>
+  <si>
+    <t>97987698076</t>
+  </si>
+  <si>
+    <t>Ramesh Saharan</t>
+  </si>
+  <si>
+    <t>rasaharan@deloitte.com</t>
+  </si>
+  <si>
+    <t>Will start working next week</t>
+  </si>
+  <si>
+    <t>8746848938</t>
+  </si>
+  <si>
     <t>UserID</t>
   </si>
   <si>
@@ -1533,39 +1566,39 @@
     <t>Admin@123</t>
   </si>
   <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>User@123</t>
+  </si>
+  <si>
     <t>User</t>
   </si>
   <si>
-    <t>TRUE</t>
-  </si>
-  <si>
-    <t>User@123</t>
-  </si>
-  <si>
     <t>kmullangi1@deloitte.com</t>
   </si>
   <si>
     <t>Admin2@456</t>
   </si>
   <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>ropatil@deloitte.com</t>
-  </si>
-  <si>
-    <t>Ropat@97</t>
+    <t>Plks@2000</t>
+  </si>
+  <si>
+    <t>Admin@789</t>
+  </si>
+  <si>
+    <t>pefernandes2@deloitte.com</t>
+  </si>
+  <si>
+    <t>Pearlfer@96</t>
   </si>
   <si>
     <t>FALSE</t>
   </si>
   <si>
-    <t>Plks@2000</t>
-  </si>
-  <si>
-    <t>Admin@789</t>
-  </si>
-  <si>
     <t>StepID</t>
   </si>
   <si>
@@ -1650,79 +1683,79 @@
     <t>CompletedDate</t>
   </si>
   <si>
+    <t>NotStarted</t>
+  </si>
+  <si>
+    <t>2026-09-05</t>
+  </si>
+  <si>
+    <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>2026-09-08</t>
+  </si>
+  <si>
+    <t>InProgress</t>
+  </si>
+  <si>
+    <t>CandidateId</t>
+  </si>
+  <si>
+    <t>Reason</t>
+  </si>
+  <si>
+    <t>.Net Dev</t>
+  </si>
+  <si>
+    <t>Client Escalation</t>
+  </si>
+  <si>
+    <t>Late to setup VDI</t>
+  </si>
+  <si>
+    <t>Contract Ended</t>
+  </si>
+  <si>
+    <t>Did not Joined</t>
+  </si>
+  <si>
+    <t>TrainingID</t>
+  </si>
+  <si>
+    <t>Domain</t>
+  </si>
+  <si>
+    <t>DueDate</t>
+  </si>
+  <si>
+    <t>DataDog</t>
+  </si>
+  <si>
+    <t>AKS</t>
+  </si>
+  <si>
+    <t>ROVO</t>
+  </si>
+  <si>
+    <t>2026-10-30</t>
+  </si>
+  <si>
     <t>2026-09-01</t>
   </si>
   <si>
-    <t>2026-09-05</t>
-  </si>
-  <si>
-    <t>2026-09-04</t>
-  </si>
-  <si>
-    <t>2026-09-07</t>
-  </si>
-  <si>
-    <t>NotStarted</t>
-  </si>
-  <si>
-    <t>InProgress</t>
-  </si>
-  <si>
-    <t>CandidateId</t>
-  </si>
-  <si>
-    <t>Reason</t>
-  </si>
-  <si>
-    <t>.Net Dev</t>
-  </si>
-  <si>
-    <t>Client Escalation</t>
-  </si>
-  <si>
-    <t>Ganesh Mundhe</t>
-  </si>
-  <si>
-    <t>Cloud Admin</t>
-  </si>
-  <si>
-    <t>Contract End</t>
-  </si>
-  <si>
-    <t>Hari Gokhale</t>
-  </si>
-  <si>
-    <t>harryG@deloitte.com</t>
-  </si>
-  <si>
-    <t>Not Joined</t>
-  </si>
-  <si>
-    <t>TrainingID</t>
-  </si>
-  <si>
-    <t>Domain</t>
-  </si>
-  <si>
-    <t>DueDate</t>
-  </si>
-  <si>
-    <t>DataDog</t>
-  </si>
-  <si>
-    <t>AKS</t>
-  </si>
-  <si>
-    <t>ROVO</t>
-  </si>
-  <si>
-    <t>2026-10-30</t>
-  </si>
-  <si>
     <t>Github Copilot</t>
   </si>
   <si>
     <t>2026-09-30</t>
+  </si>
+  <si>
+    <t>2026-08-31</t>
+  </si>
+  <si>
+    <t>2026-09-03</t>
+  </si>
+  <si>
+    <t>2026-09-02</t>
   </si>
   <si>
     <t>Project name</t>
@@ -3742,7 +3775,7 @@
     <xf numFmtId="0" applyNumberFormat="0" fontId="1" applyFont="1" fillId="0" applyFill="0" borderId="0" applyBorder="0" applyProtection="0" applyAlignment="0"/>
     <xf numFmtId="9" applyNumberFormat="1" fontId="2" applyFont="0" fillId="0" applyFill="0" borderId="0" applyBorder="0" applyProtection="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="339">
+  <cellXfs count="338">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" applyFill="1" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" applyFont="1" fillId="0" borderId="0" xfId="1"/>
@@ -4404,9 +4437,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" applyNumberFormat="1" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -7407,7 +7437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{358897FF-3897-4B6D-8A0F-DEA84C78DC28}">
-  <dimension ref="A1:AI101"/>
+  <dimension ref="A1:AI103"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.54296875" customWidth="1"/>
@@ -16877,11 +16907,17 @@
       <c r="I101" s="0" t="s">
         <v>439</v>
       </c>
+      <c r="K101" s="0" t="s">
+        <v>440</v>
+      </c>
+      <c r="L101" s="0" t="s">
+        <v>127</v>
+      </c>
       <c r="M101" s="0" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="N101" s="0" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="O101" s="0" t="s">
         <v>42</v>
@@ -16893,22 +16929,140 @@
         <v>126</v>
       </c>
       <c r="U101" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="V101" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="W101" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB101" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE101" s="0" t="s">
+        <v>443</v>
+      </c>
+      <c r="AG101" s="0" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="0">
+        <v>101</v>
+      </c>
+      <c r="B102" s="0" t="s">
+        <v>445</v>
+      </c>
+      <c r="C102" s="0" t="s">
+        <v>446</v>
+      </c>
+      <c r="D102" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="E102" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="G102" s="0" t="s">
+        <v>197</v>
+      </c>
+      <c r="I102" s="0" t="s">
+        <v>439</v>
+      </c>
+      <c r="K102" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="L102" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="M102" s="0" t="s">
+        <v>441</v>
+      </c>
+      <c r="N102" s="0" t="s">
+        <v>442</v>
+      </c>
+      <c r="O102" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="P102" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q102" s="0" t="s">
+        <v>448</v>
+      </c>
+      <c r="U102" s="0" t="s">
         <v>127</v>
       </c>
-      <c r="V101" s="0" t="s">
+      <c r="V102" s="0" t="s">
         <v>127</v>
       </c>
-      <c r="W101" s="0" t="s">
+      <c r="W102" s="0" t="s">
         <v>127</v>
       </c>
-      <c r="AB101" s="0" t="s">
+      <c r="AB102" s="0" t="s">
         <v>127</v>
       </c>
-      <c r="AE101" s="0" t="s">
+      <c r="AE102" s="0" t="s">
+        <v>449</v>
+      </c>
+      <c r="AG102" s="0" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="0">
+        <v>102</v>
+      </c>
+      <c r="B103" s="0" t="s">
+        <v>451</v>
+      </c>
+      <c r="C103" s="0" t="s">
+        <v>452</v>
+      </c>
+      <c r="D103" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="E103" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="G103" s="0" t="s">
+        <v>197</v>
+      </c>
+      <c r="I103" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="M103" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="N103" s="0" t="s">
         <v>442</v>
       </c>
-      <c r="AG101" s="0" t="s">
-        <v>443</v>
+      <c r="O103" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="P103" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q103" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="U103" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="V103" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="W103" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="AB103" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="AE103" s="0" t="s">
+        <v>453</v>
+      </c>
+      <c r="AG103" s="0" t="s">
+        <v>454</v>
       </c>
     </row>
   </sheetData>
@@ -17085,21 +17239,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>627</v>
+        <v>638</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>629</v>
+        <v>640</v>
       </c>
       <c r="B2" s="0" t="s">
         <v>50</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
     </row>
     <row r="3">
@@ -17192,7 +17346,7 @@
     </row>
     <row r="11">
       <c r="A11" s="80" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
       <c r="B11" s="78">
         <v>84</v>
@@ -17220,22 +17374,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="77" t="s">
-        <v>631</v>
+        <v>642</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="78" t="s">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="B2" s="78" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
       <c r="C2" s="78"/>
       <c r="D2" s="78"/>
     </row>
     <row r="3">
       <c r="A3" s="78" t="s">
-        <v>629</v>
+        <v>640</v>
       </c>
       <c r="B3" s="78" t="s">
         <v>127</v>
@@ -17244,7 +17398,7 @@
         <v>45</v>
       </c>
       <c r="D3" s="78" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
     </row>
     <row r="4">
@@ -17407,7 +17561,7 @@
     </row>
     <row r="17">
       <c r="A17" s="78" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
       <c r="B17" s="78">
         <v>6</v>
@@ -17426,20 +17580,20 @@
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>633</v>
+        <v>644</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="77" t="s">
-        <v>634</v>
+        <v>645</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="78" t="s">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="B23" s="78" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
       <c r="C23" s="78"/>
       <c r="D23" s="78"/>
@@ -17447,7 +17601,7 @@
     </row>
     <row r="24">
       <c r="A24" s="78" t="s">
-        <v>629</v>
+        <v>640</v>
       </c>
       <c r="B24" s="78" t="s">
         <v>83</v>
@@ -17459,7 +17613,7 @@
         <v>61</v>
       </c>
       <c r="E24" s="78" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
     </row>
     <row r="25">
@@ -17643,7 +17797,7 @@
     </row>
     <row r="38">
       <c r="A38" s="78" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
       <c r="B38" s="78">
         <v>24</v>
@@ -17660,63 +17814,63 @@
     </row>
     <row r="41">
       <c r="A41" s="78" t="s">
-        <v>635</v>
+        <v>646</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>636</v>
+        <v>647</v>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="0" t="s">
-        <v>637</v>
+        <v>648</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="0" t="s">
-        <v>638</v>
+        <v>649</v>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="0" t="s">
-        <v>639</v>
+        <v>650</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="79" t="s">
-        <v>640</v>
+        <v>651</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="0" t="s">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="0" t="s">
-        <v>629</v>
+        <v>640</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>641</v>
+        <v>652</v>
       </c>
       <c r="C51" s="0" t="s">
         <v>36</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>642</v>
+        <v>653</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>643</v>
+        <v>654</v>
       </c>
       <c r="F51" s="0" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="80" t="s">
-        <v>644</v>
+        <v>655</v>
       </c>
       <c r="B52" s="0">
         <v>5</v>
@@ -17733,7 +17887,7 @@
     </row>
     <row r="53">
       <c r="A53" s="80" t="s">
-        <v>645</v>
+        <v>656</v>
       </c>
       <c r="C53" s="0">
         <v>8</v>
@@ -17744,7 +17898,7 @@
     </row>
     <row r="54">
       <c r="A54" s="80" t="s">
-        <v>646</v>
+        <v>657</v>
       </c>
       <c r="B54" s="0">
         <v>1</v>
@@ -17761,12 +17915,12 @@
     </row>
     <row r="55">
       <c r="A55" s="80" t="s">
-        <v>643</v>
+        <v>654</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="80" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
       <c r="B56" s="0">
         <v>6</v>
@@ -17783,7 +17937,7 @@
     </row>
     <row r="59">
       <c r="A59" s="70" t="s">
-        <v>647</v>
+        <v>658</v>
       </c>
       <c r="B59" s="71"/>
       <c r="C59" s="71"/>
@@ -17792,19 +17946,19 @@
     </row>
     <row r="60">
       <c r="A60" s="70" t="s">
-        <v>648</v>
+        <v>659</v>
       </c>
       <c r="B60" s="70" t="s">
-        <v>610</v>
+        <v>621</v>
       </c>
       <c r="C60" s="70" t="s">
-        <v>611</v>
+        <v>622</v>
       </c>
       <c r="D60" s="70" t="s">
-        <v>612</v>
+        <v>623</v>
       </c>
       <c r="E60" s="70" t="s">
-        <v>613</v>
+        <v>624</v>
       </c>
       <c r="F60" s="77"/>
     </row>
@@ -17813,7 +17967,7 @@
         <v>38</v>
       </c>
       <c r="B61" s="71" t="s">
-        <v>614</v>
+        <v>625</v>
       </c>
       <c r="C61" s="71">
         <v>12</v>
@@ -17828,7 +17982,7 @@
     <row r="62">
       <c r="A62" s="325"/>
       <c r="B62" s="71" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="C62" s="71">
         <v>9</v>
@@ -17843,7 +17997,7 @@
     <row r="63">
       <c r="A63" s="326"/>
       <c r="B63" s="71" t="s">
-        <v>512</v>
+        <v>520</v>
       </c>
       <c r="C63" s="71">
         <v>27</v>
@@ -17896,15 +18050,15 @@
         <v>4</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>649</v>
+        <v>660</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>629</v>
+        <v>640</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>650</v>
+        <v>661</v>
       </c>
     </row>
     <row r="4">
@@ -18005,7 +18159,7 @@
     </row>
     <row r="16">
       <c r="A16" s="80" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
       <c r="B16" s="0">
         <v>104</v>
@@ -18031,10 +18185,10 @@
         <v>12</v>
       </c>
       <c r="B1" s="291" t="s">
-        <v>651</v>
+        <v>662</v>
       </c>
       <c r="C1" s="291" t="s">
-        <v>652</v>
+        <v>663</v>
       </c>
     </row>
     <row r="2" ht="29">
@@ -18042,10 +18196,10 @@
         <v>198</v>
       </c>
       <c r="B2" s="293" t="s">
-        <v>653</v>
+        <v>664</v>
       </c>
       <c r="C2" s="294" t="s">
-        <v>654</v>
+        <v>665</v>
       </c>
     </row>
     <row r="3">
@@ -18053,10 +18207,10 @@
         <v>110</v>
       </c>
       <c r="B3" s="295" t="s">
-        <v>655</v>
+        <v>666</v>
       </c>
       <c r="C3" s="294" t="s">
-        <v>656</v>
+        <v>667</v>
       </c>
     </row>
     <row r="4" ht="29">
@@ -18064,32 +18218,32 @@
         <v>141</v>
       </c>
       <c r="B4" s="293" t="s">
-        <v>653</v>
+        <v>664</v>
       </c>
       <c r="C4" s="294" t="s">
-        <v>657</v>
+        <v>668</v>
       </c>
     </row>
     <row r="5" ht="58">
       <c r="A5" s="292" t="s">
-        <v>658</v>
+        <v>669</v>
       </c>
       <c r="B5" s="293" t="s">
-        <v>653</v>
+        <v>664</v>
       </c>
       <c r="C5" s="294" t="s">
-        <v>659</v>
+        <v>670</v>
       </c>
     </row>
     <row r="6" ht="29">
       <c r="A6" s="293" t="s">
-        <v>660</v>
+        <v>671</v>
       </c>
       <c r="B6" s="293" t="s">
-        <v>655</v>
+        <v>666</v>
       </c>
       <c r="C6" s="294" t="s">
-        <v>661</v>
+        <v>672</v>
       </c>
     </row>
     <row r="7">
@@ -18097,10 +18251,10 @@
         <v>58</v>
       </c>
       <c r="B7" s="293" t="s">
-        <v>614</v>
+        <v>625</v>
       </c>
       <c r="C7" s="294" t="s">
-        <v>662</v>
+        <v>673</v>
       </c>
     </row>
     <row r="8">
@@ -18108,7 +18262,7 @@
         <v>174</v>
       </c>
       <c r="B8" s="297" t="s">
-        <v>653</v>
+        <v>664</v>
       </c>
       <c r="C8" s="296" t="s">
         <v>172</v>
@@ -18119,10 +18273,10 @@
         <v>113</v>
       </c>
       <c r="B9" s="297" t="s">
-        <v>653</v>
+        <v>664</v>
       </c>
       <c r="C9" s="296" t="s">
-        <v>663</v>
+        <v>674</v>
       </c>
     </row>
   </sheetData>
@@ -18142,18 +18296,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="288" t="s">
-        <v>664</v>
+        <v>675</v>
       </c>
       <c r="B1" s="288" t="s">
-        <v>665</v>
+        <v>676</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="289" t="s">
-        <v>666</v>
+        <v>677</v>
       </c>
       <c r="B2" s="290" t="s">
-        <v>667</v>
+        <v>678</v>
       </c>
     </row>
   </sheetData>
@@ -18179,19 +18333,19 @@
   <sheetData>
     <row r="1" ht="39">
       <c r="A1" s="298" t="s">
-        <v>668</v>
+        <v>679</v>
       </c>
       <c r="B1" s="299" t="s">
-        <v>669</v>
+        <v>680</v>
       </c>
       <c r="C1" s="299" t="s">
-        <v>670</v>
+        <v>681</v>
       </c>
       <c r="D1" s="299" t="s">
-        <v>671</v>
+        <v>682</v>
       </c>
       <c r="E1" s="300" t="s">
-        <v>672</v>
+        <v>683</v>
       </c>
     </row>
     <row r="2" ht="247" customHeight="1">
@@ -18199,16 +18353,16 @@
         <v>198</v>
       </c>
       <c r="B2" s="329" t="s">
-        <v>673</v>
+        <v>684</v>
       </c>
       <c r="C2" s="329">
         <v>2</v>
       </c>
       <c r="D2" s="331" t="s">
-        <v>674</v>
+        <v>685</v>
       </c>
       <c r="E2" s="301" t="s">
-        <v>675</v>
+        <v>686</v>
       </c>
     </row>
     <row r="3" ht="26.5">
@@ -18217,22 +18371,22 @@
       <c r="C3" s="330"/>
       <c r="D3" s="332"/>
       <c r="E3" s="302" t="s">
-        <v>676</v>
+        <v>687</v>
       </c>
     </row>
     <row r="4" ht="156.5">
       <c r="A4" s="328"/>
       <c r="B4" s="303" t="s">
-        <v>677</v>
+        <v>688</v>
       </c>
       <c r="C4" s="303">
         <v>2</v>
       </c>
       <c r="D4" s="304" t="s">
-        <v>678</v>
+        <v>689</v>
       </c>
       <c r="E4" s="302" t="s">
-        <v>679</v>
+        <v>690</v>
       </c>
     </row>
     <row r="5" ht="39.5">
@@ -18246,10 +18400,10 @@
         <v>3</v>
       </c>
       <c r="D5" s="305" t="s">
-        <v>680</v>
+        <v>691</v>
       </c>
       <c r="E5" s="302" t="s">
-        <v>681</v>
+        <v>692</v>
       </c>
     </row>
     <row r="6" ht="65.5">
@@ -18257,15 +18411,15 @@
       <c r="B6" s="330"/>
       <c r="C6" s="330"/>
       <c r="D6" s="306" t="s">
-        <v>682</v>
+        <v>693</v>
       </c>
       <c r="E6" s="307" t="s">
-        <v>683</v>
+        <v>694</v>
       </c>
     </row>
     <row r="7" ht="52.5">
       <c r="A7" s="327" t="s">
-        <v>684</v>
+        <v>695</v>
       </c>
       <c r="B7" s="329" t="s">
         <v>96</v>
@@ -18274,10 +18428,10 @@
         <v>3</v>
       </c>
       <c r="D7" s="305" t="s">
-        <v>685</v>
+        <v>696</v>
       </c>
       <c r="E7" s="301" t="s">
-        <v>686</v>
+        <v>697</v>
       </c>
     </row>
     <row r="8" ht="65.5">
@@ -18285,10 +18439,10 @@
       <c r="B8" s="336"/>
       <c r="C8" s="336"/>
       <c r="D8" s="308" t="s">
-        <v>687</v>
+        <v>698</v>
       </c>
       <c r="E8" s="309" t="s">
-        <v>688</v>
+        <v>699</v>
       </c>
     </row>
     <row r="9" ht="39.5">
@@ -18296,13 +18450,13 @@
       <c r="B9" s="330"/>
       <c r="C9" s="330"/>
       <c r="D9" s="306" t="s">
-        <v>689</v>
+        <v>700</v>
       </c>
       <c r="E9" s="310"/>
     </row>
     <row r="10" ht="273" customHeight="1">
       <c r="A10" s="327" t="s">
-        <v>690</v>
+        <v>701</v>
       </c>
       <c r="B10" s="329" t="s">
         <v>87</v>
@@ -18311,10 +18465,10 @@
         <v>4</v>
       </c>
       <c r="D10" s="334" t="s">
-        <v>691</v>
+        <v>702</v>
       </c>
       <c r="E10" s="301" t="s">
-        <v>692</v>
+        <v>703</v>
       </c>
     </row>
     <row r="11" ht="26.5">
@@ -18323,7 +18477,7 @@
       <c r="C11" s="330"/>
       <c r="D11" s="335"/>
       <c r="E11" s="307" t="s">
-        <v>693</v>
+        <v>704</v>
       </c>
     </row>
     <row r="12" ht="65.5">
@@ -18337,10 +18491,10 @@
         <v>2</v>
       </c>
       <c r="D12" s="304" t="s">
-        <v>694</v>
+        <v>705</v>
       </c>
       <c r="E12" s="312" t="s">
-        <v>695</v>
+        <v>706</v>
       </c>
     </row>
   </sheetData>
@@ -18376,26 +18530,26 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="275" t="s">
-        <v>696</v>
+        <v>707</v>
       </c>
       <c r="B1" s="276" t="s">
-        <v>665</v>
+        <v>676</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="71" t="s">
-        <v>697</v>
+        <v>708</v>
       </c>
       <c r="B2" s="101" t="s">
-        <v>698</v>
+        <v>709</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="71" t="s">
-        <v>699</v>
+        <v>710</v>
       </c>
       <c r="B3" s="101" t="s">
-        <v>700</v>
+        <v>711</v>
       </c>
     </row>
   </sheetData>
@@ -18420,104 +18574,104 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="77" t="s">
-        <v>701</v>
+        <v>712</v>
       </c>
       <c r="B1" s="77" t="s">
-        <v>702</v>
+        <v>713</v>
       </c>
       <c r="C1" s="77" t="s">
-        <v>703</v>
+        <v>714</v>
       </c>
       <c r="D1" s="77" t="s">
-        <v>704</v>
+        <v>715</v>
       </c>
       <c r="E1" s="77" t="s">
-        <v>705</v>
+        <v>716</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>706</v>
+        <v>717</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>707</v>
+        <v>718</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>708</v>
+        <v>719</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>709</v>
+        <v>720</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>710</v>
+        <v>721</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>706</v>
+        <v>717</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>711</v>
+        <v>722</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>712</v>
+        <v>723</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>714</v>
+        <v>725</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>715</v>
+        <v>726</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>716</v>
+        <v>727</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>717</v>
+        <v>728</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>709</v>
+        <v>720</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>710</v>
+        <v>721</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>715</v>
+        <v>726</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>718</v>
+        <v>729</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>719</v>
+        <v>730</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>720</v>
+        <v>731</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>714</v>
+        <v>725</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>715</v>
+        <v>726</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>721</v>
+        <v>732</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>722</v>
+        <v>733</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>723</v>
+        <v>734</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>714</v>
+        <v>725</v>
       </c>
     </row>
   </sheetData>
@@ -18547,53 +18701,53 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="77" t="s">
-        <v>701</v>
+        <v>712</v>
       </c>
       <c r="B1" s="77" t="s">
-        <v>702</v>
+        <v>713</v>
       </c>
       <c r="C1" s="77" t="s">
-        <v>703</v>
+        <v>714</v>
       </c>
       <c r="D1" s="77" t="s">
-        <v>704</v>
+        <v>715</v>
       </c>
       <c r="E1" s="77" t="s">
-        <v>705</v>
+        <v>716</v>
       </c>
     </row>
     <row r="2" ht="101.5">
       <c r="A2" s="0" t="s">
-        <v>706</v>
+        <v>717</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>724</v>
+        <v>735</v>
       </c>
       <c r="C2" s="277" t="s">
-        <v>725</v>
+        <v>736</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>726</v>
+        <v>737</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>727</v>
+        <v>738</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>728</v>
+        <v>739</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>729</v>
+        <v>740</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>720</v>
+        <v>731</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>727</v>
+        <v>738</v>
       </c>
     </row>
   </sheetData>
@@ -18613,62 +18767,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="77" t="s">
-        <v>701</v>
+        <v>712</v>
       </c>
       <c r="B1" s="77" t="s">
-        <v>702</v>
+        <v>713</v>
       </c>
       <c r="C1" s="77" t="s">
-        <v>703</v>
+        <v>714</v>
       </c>
       <c r="D1" s="77" t="s">
-        <v>704</v>
+        <v>715</v>
       </c>
       <c r="E1" s="77" t="s">
-        <v>705</v>
+        <v>716</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>728</v>
+        <v>739</v>
       </c>
       <c r="C2" s="278" t="s">
-        <v>730</v>
+        <v>741</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>728</v>
+        <v>739</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>510</v>
+        <v>517</v>
       </c>
       <c r="C3" s="278" t="s">
-        <v>731</v>
+        <v>742</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>728</v>
+        <v>739</v>
       </c>
       <c r="C4" s="278" t="s">
-        <v>732</v>
+        <v>743</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>733</v>
+        <v>744</v>
       </c>
       <c r="C5" s="278" t="s">
-        <v>734</v>
+        <v>745</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>733</v>
+        <v>744</v>
       </c>
       <c r="C6" s="278" t="s">
-        <v>735</v>
+        <v>746</v>
       </c>
     </row>
   </sheetData>
@@ -18695,19 +18849,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>444</v>
+        <v>455</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>445</v>
+        <v>456</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>446</v>
+        <v>457</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>447</v>
+        <v>458</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
     </row>
     <row r="2">
@@ -18718,13 +18872,13 @@
         <v>161</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>449</v>
+        <v>460</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>450</v>
+        <v>461</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>451</v>
+        <v>462</v>
       </c>
     </row>
     <row r="3">
@@ -18735,13 +18889,13 @@
         <v>351</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>452</v>
+        <v>463</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>450</v>
+        <v>464</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>451</v>
+        <v>462</v>
       </c>
     </row>
     <row r="4">
@@ -18749,67 +18903,67 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>453</v>
+        <v>465</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>454</v>
+        <v>466</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>451</v>
+        <v>462</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>456</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>457</v>
+        <v>435</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>467</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>450</v>
+        <v>464</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>435</v>
+        <v>91</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>459</v>
+        <v>468</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>450</v>
+        <v>461</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>451</v>
+        <v>462</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>91</v>
+        <v>469</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>451</v>
+        <v>471</v>
       </c>
     </row>
   </sheetData>
@@ -18820,7 +18974,6 @@
     <hyperlink ref="C3" r:id="rId4"/>
     <hyperlink ref="B4" r:id="rId5"/>
     <hyperlink ref="C4" r:id="rId6"/>
-    <hyperlink ref="C5" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
@@ -18839,68 +18992,68 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="77" t="s">
-        <v>701</v>
+        <v>712</v>
       </c>
       <c r="B1" s="77" t="s">
-        <v>702</v>
+        <v>713</v>
       </c>
       <c r="C1" s="77" t="s">
-        <v>703</v>
+        <v>714</v>
       </c>
       <c r="D1" s="77" t="s">
-        <v>704</v>
+        <v>715</v>
       </c>
       <c r="E1" s="77" t="s">
-        <v>705</v>
+        <v>716</v>
       </c>
     </row>
     <row r="2" ht="43.5">
       <c r="A2" s="337" t="s">
-        <v>706</v>
+        <v>717</v>
       </c>
       <c r="B2" s="173" t="s">
-        <v>736</v>
+        <v>747</v>
       </c>
       <c r="C2" s="277" t="s">
-        <v>737</v>
+        <v>748</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>710</v>
+        <v>721</v>
       </c>
     </row>
     <row r="3" ht="29">
       <c r="A3" s="337"/>
       <c r="B3" s="173" t="s">
-        <v>738</v>
+        <v>749</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>739</v>
+        <v>750</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>740</v>
+        <v>751</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>710</v>
+        <v>721</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>741</v>
+        <v>752</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>742</v>
+        <v>753</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>743</v>
+        <v>754</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>726</v>
+        <v>737</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>710</v>
+        <v>721</v>
       </c>
     </row>
     <row r="6">
@@ -18908,19 +19061,19 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>744</v>
+        <v>755</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>745</v>
+        <v>756</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>746</v>
+        <v>757</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>710</v>
+        <v>721</v>
       </c>
     </row>
   </sheetData>
@@ -18949,98 +19102,98 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="275" t="s">
-        <v>664</v>
+        <v>675</v>
       </c>
       <c r="B1" s="77" t="s">
-        <v>665</v>
+        <v>676</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="279" t="s">
-        <v>748</v>
+        <v>759</v>
       </c>
       <c r="B2" s="280" t="s">
-        <v>749</v>
+        <v>760</v>
       </c>
     </row>
     <row r="3" ht="43.5">
       <c r="A3" s="281" t="s">
-        <v>750</v>
+        <v>761</v>
       </c>
       <c r="B3" s="282" t="s">
-        <v>751</v>
+        <v>762</v>
       </c>
     </row>
     <row r="4" ht="43.5">
       <c r="A4" s="281" t="s">
-        <v>752</v>
+        <v>763</v>
       </c>
       <c r="B4" s="282" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
     </row>
     <row r="5" ht="101.5">
       <c r="A5" s="281" t="s">
-        <v>754</v>
+        <v>765</v>
       </c>
       <c r="B5" s="283" t="s">
-        <v>755</v>
+        <v>766</v>
       </c>
     </row>
     <row r="6" ht="29">
       <c r="A6" s="281" t="s">
-        <v>756</v>
+        <v>767</v>
       </c>
       <c r="B6" s="282" t="s">
-        <v>757</v>
+        <v>768</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="279" t="s">
-        <v>758</v>
+        <v>769</v>
       </c>
       <c r="B7" s="280" t="s">
-        <v>759</v>
+        <v>770</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="279" t="s">
-        <v>760</v>
+        <v>771</v>
       </c>
       <c r="B8" s="280" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
     </row>
     <row r="9" ht="72.5">
       <c r="A9" s="281" t="s">
-        <v>762</v>
+        <v>773</v>
       </c>
       <c r="B9" s="282" t="s">
-        <v>763</v>
+        <v>774</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="279" t="s">
-        <v>764</v>
+        <v>775</v>
       </c>
       <c r="B10" s="280" t="s">
-        <v>765</v>
+        <v>776</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="284" t="s">
-        <v>766</v>
+        <v>777</v>
       </c>
       <c r="B11" s="280" t="s">
-        <v>767</v>
+        <v>778</v>
       </c>
     </row>
     <row r="12" ht="58">
       <c r="A12" s="285" t="s">
-        <v>768</v>
+        <v>779</v>
       </c>
       <c r="B12" s="282" t="s">
-        <v>769</v>
+        <v>780</v>
       </c>
     </row>
   </sheetData>
@@ -19073,26 +19226,26 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="67" t="s">
-        <v>665</v>
+        <v>676</v>
       </c>
       <c r="B1" s="67" t="s">
-        <v>770</v>
+        <v>781</v>
       </c>
     </row>
     <row r="2" ht="43.5">
       <c r="A2" s="286" t="s">
-        <v>737</v>
+        <v>748</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>771</v>
+        <v>782</v>
       </c>
     </row>
     <row r="3" ht="43.5">
       <c r="A3" s="286" t="s">
-        <v>772</v>
+        <v>783</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>773</v>
+        <v>784</v>
       </c>
     </row>
   </sheetData>
@@ -19116,50 +19269,50 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="77" t="s">
-        <v>665</v>
+        <v>676</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>705</v>
+        <v>716</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>774</v>
+        <v>785</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>775</v>
+        <v>786</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>776</v>
+        <v>787</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>777</v>
+        <v>788</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>778</v>
+        <v>789</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>779</v>
+        <v>790</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>780</v>
+        <v>791</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>781</v>
+        <v>792</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>782</v>
+        <v>793</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>783</v>
+        <v>794</v>
       </c>
     </row>
   </sheetData>
@@ -19186,34 +19339,34 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="287" t="s">
-        <v>664</v>
+        <v>675</v>
       </c>
       <c r="B1" s="276" t="s">
-        <v>665</v>
+        <v>676</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="114" t="s">
-        <v>784</v>
+        <v>795</v>
       </c>
       <c r="B2" s="101" t="s">
-        <v>785</v>
+        <v>796</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="71" t="s">
-        <v>786</v>
+        <v>797</v>
       </c>
       <c r="B3" s="101" t="s">
-        <v>787</v>
+        <v>798</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="71" t="s">
-        <v>788</v>
+        <v>799</v>
       </c>
       <c r="B4" s="101" t="s">
-        <v>789</v>
+        <v>800</v>
       </c>
     </row>
   </sheetData>
@@ -19240,19 +19393,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>461</v>
+        <v>472</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>462</v>
+        <v>473</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>463</v>
+        <v>474</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>464</v>
+        <v>475</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>465</v>
+        <v>476</v>
       </c>
     </row>
     <row r="2">
@@ -19263,13 +19416,13 @@
         <v>169</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>466</v>
+        <v>477</v>
       </c>
       <c r="D2" s="0">
         <v>1</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>467</v>
+        <v>478</v>
       </c>
     </row>
     <row r="3">
@@ -19280,13 +19433,13 @@
         <v>169</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>468</v>
+        <v>479</v>
       </c>
       <c r="D3" s="0">
         <v>2</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
     </row>
     <row r="4">
@@ -19297,13 +19450,13 @@
         <v>169</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="D4" s="0">
         <v>3</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>471</v>
+        <v>482</v>
       </c>
     </row>
     <row r="5">
@@ -19314,13 +19467,13 @@
         <v>169</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>472</v>
+        <v>483</v>
       </c>
       <c r="D5" s="0">
         <v>4</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>473</v>
+        <v>484</v>
       </c>
     </row>
     <row r="6">
@@ -19328,16 +19481,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
       <c r="D6" s="0">
         <v>1</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>476</v>
+        <v>487</v>
       </c>
     </row>
     <row r="7">
@@ -19345,16 +19498,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>468</v>
+        <v>479</v>
       </c>
       <c r="D7" s="0">
         <v>2</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
     </row>
     <row r="8">
@@ -19362,16 +19515,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="D8" s="0">
         <v>3</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>471</v>
+        <v>482</v>
       </c>
     </row>
     <row r="9">
@@ -19379,16 +19532,16 @@
         <v>9</v>
       </c>
       <c r="B9" s="0" t="s">
+        <v>488</v>
+      </c>
+      <c r="C9" s="0" t="s">
         <v>477</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>466</v>
       </c>
       <c r="D9" s="0">
         <v>1</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>467</v>
+        <v>478</v>
       </c>
     </row>
     <row r="10">
@@ -19396,16 +19549,16 @@
         <v>10</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>477</v>
+        <v>488</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>468</v>
+        <v>479</v>
       </c>
       <c r="D10" s="0">
         <v>2</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
     </row>
     <row r="11">
@@ -19413,16 +19566,16 @@
         <v>11</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>477</v>
+        <v>488</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="D11" s="0">
         <v>3</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>471</v>
+        <v>482</v>
       </c>
     </row>
     <row r="12">
@@ -19430,16 +19583,16 @@
         <v>12</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>477</v>
+        <v>488</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>472</v>
+        <v>483</v>
       </c>
       <c r="D12" s="0">
         <v>4</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>473</v>
+        <v>484</v>
       </c>
     </row>
     <row r="13">
@@ -19447,16 +19600,16 @@
         <v>13</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>466</v>
+        <v>477</v>
       </c>
       <c r="D13" s="0">
         <v>1</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>467</v>
+        <v>478</v>
       </c>
     </row>
     <row r="14">
@@ -19464,16 +19617,16 @@
         <v>14</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>468</v>
+        <v>479</v>
       </c>
       <c r="D14" s="0">
         <v>2</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
     </row>
     <row r="15">
@@ -19481,16 +19634,16 @@
         <v>15</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="D15" s="0">
         <v>3</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>471</v>
+        <v>482</v>
       </c>
     </row>
     <row r="16">
@@ -19498,16 +19651,16 @@
         <v>16</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>472</v>
+        <v>483</v>
       </c>
       <c r="D16" s="0">
         <v>4</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>473</v>
+        <v>484</v>
       </c>
     </row>
     <row r="17">
@@ -19515,16 +19668,16 @@
         <v>17</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>479</v>
+        <v>490</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>466</v>
+        <v>477</v>
       </c>
       <c r="D17" s="0">
         <v>1</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>467</v>
+        <v>478</v>
       </c>
     </row>
     <row r="18">
@@ -19532,16 +19685,16 @@
         <v>18</v>
       </c>
       <c r="B18" s="0" t="s">
+        <v>490</v>
+      </c>
+      <c r="C18" s="0" t="s">
         <v>479</v>
-      </c>
-      <c r="C18" s="0" t="s">
-        <v>468</v>
       </c>
       <c r="D18" s="0">
         <v>2</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
     </row>
     <row r="19">
@@ -19549,16 +19702,16 @@
         <v>19</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>479</v>
+        <v>490</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="D19" s="0">
         <v>3</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>471</v>
+        <v>482</v>
       </c>
     </row>
     <row r="20">
@@ -19566,16 +19719,16 @@
         <v>20</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>479</v>
+        <v>490</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>472</v>
+        <v>483</v>
       </c>
       <c r="D20" s="0">
         <v>4</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>473</v>
+        <v>484</v>
       </c>
     </row>
     <row r="21">
@@ -19583,16 +19736,16 @@
         <v>21</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>480</v>
+        <v>491</v>
       </c>
       <c r="D21" s="0">
         <v>4</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>481</v>
+        <v>492</v>
       </c>
     </row>
     <row r="22">
@@ -19600,16 +19753,16 @@
         <v>22</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>482</v>
+        <v>493</v>
       </c>
       <c r="D22" s="0">
         <v>5</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>483</v>
+        <v>494</v>
       </c>
     </row>
     <row r="23">
@@ -19620,13 +19773,13 @@
         <v>206</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
       <c r="D23" s="0">
         <v>1</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>484</v>
+        <v>495</v>
       </c>
     </row>
   </sheetData>
@@ -19637,7 +19790,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89F9B618-8BC8-49DD-B7A7-74400FF462D0}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.36328125" customWidth="1"/>
@@ -19648,106 +19801,112 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>485</v>
+        <v>496</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>486</v>
+        <v>497</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>461</v>
+        <v>472</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>487</v>
+        <v>498</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>488</v>
+        <v>499</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" s="0">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C2" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>61</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>489</v>
+        <v>500</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" s="0">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="C3" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>320</v>
+        <v>500</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" s="0">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C4" s="0">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>320</v>
+        <v>61</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>501</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B5" s="0">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="C5" s="0">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D5" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="E5" s="338">
-        <v>46239</v>
+      <c r="E5" s="0" t="s">
+        <v>502</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B6" s="0">
-        <v>34</v>
+        <v>80</v>
       </c>
       <c r="C6" s="0">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D6" s="0" t="s">
         <v>61</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B7" s="0">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="C7" s="0">
         <v>5</v>
@@ -19756,108 +19915,74 @@
         <v>61</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>491</v>
+        <v>447</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B8" s="0">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="C8" s="0">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D8" s="0" t="s">
         <v>61</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>491</v>
+        <v>447</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B9" s="0">
         <v>25</v>
       </c>
       <c r="C9" s="0">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D9" s="0" t="s">
         <v>61</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>492</v>
+        <v>447</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B10" s="0">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C10" s="0">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D10" s="0" t="s">
         <v>61</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>492</v>
+        <v>503</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11" s="0">
         <v>25</v>
       </c>
       <c r="C11" s="0">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>61</v>
+        <v>504</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="0">
-        <v>11</v>
-      </c>
-      <c r="B12" s="0">
-        <v>25</v>
-      </c>
-      <c r="C12" s="0">
-        <v>21</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>493</v>
-      </c>
-      <c r="E12" s="0" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="0">
-        <v>12</v>
-      </c>
-      <c r="B13" s="0">
-        <v>25</v>
-      </c>
-      <c r="C13" s="0">
-        <v>22</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>494</v>
-      </c>
-      <c r="E13" s="0" t="s">
         <v>46</v>
       </c>
     </row>
@@ -19869,7 +19994,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5417B356-7CA8-4073-B5EA-2ED7E0869648}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.36328125" customWidth="1"/>
@@ -19881,7 +20006,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>495</v>
+        <v>505</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
@@ -19890,10 +20015,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>447</v>
+        <v>458</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>496</v>
+        <v>506</v>
       </c>
     </row>
     <row r="2">
@@ -19907,50 +20032,66 @@
         <v>347</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>497</v>
+        <v>507</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>498</v>
+        <v>508</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0">
-        <v>98</v>
+        <v>35</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>499</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>218</v>
+        <v>192</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>193</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>500</v>
+        <v>52</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>501</v>
+        <v>509</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0">
-        <v>131</v>
+        <v>41</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>502</v>
+        <v>217</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>503</v>
+        <v>218</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>119</v>
+        <v>439</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>504</v>
+        <v>510</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>60</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>288</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>289</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>511</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1"/>
-    <hyperlink ref="C3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
@@ -19959,7 +20100,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B14947C1-2082-4307-8EB3-961E6465F131}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.6328125" customWidth="1"/>
@@ -19972,22 +20113,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>486</v>
+        <v>497</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>506</v>
+        <v>513</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>487</v>
+        <v>498</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>507</v>
+        <v>514</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>488</v>
+        <v>499</v>
       </c>
     </row>
     <row r="2">
@@ -19998,7 +20139,7 @@
         <v>22</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>508</v>
+        <v>515</v>
       </c>
       <c r="D2" s="0" t="s">
         <v>61</v>
@@ -20018,7 +20159,7 @@
         <v>22</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="D3" s="0" t="s">
         <v>320</v>
@@ -20035,7 +20176,7 @@
         <v>22</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>510</v>
+        <v>517</v>
       </c>
       <c r="D4" s="0" t="s">
         <v>61</v>
@@ -20055,7 +20196,7 @@
         <v>78</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>508</v>
+        <v>515</v>
       </c>
       <c r="D5" s="0" t="s">
         <v>61</v>
@@ -20075,7 +20216,7 @@
         <v>87</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="D6" s="0" t="s">
         <v>320</v>
@@ -20098,10 +20239,10 @@
         <v>61</v>
       </c>
       <c r="E7" s="314" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="F7" s="314" t="s">
-        <v>489</v>
+        <v>519</v>
       </c>
     </row>
     <row r="8">
@@ -20112,13 +20253,73 @@
         <v>78</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>512</v>
+        <v>520</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>494</v>
+        <v>504</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>513</v>
+        <v>521</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0">
+        <v>94</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>517</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>500</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>522</v>
+      </c>
+      <c r="F9" s="0" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0">
+        <v>55</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>522</v>
+      </c>
+      <c r="F10" s="0" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0">
+        <v>97</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>522</v>
+      </c>
+      <c r="F11" s="0" t="s">
+        <v>524</v>
       </c>
     </row>
   </sheetData>
@@ -20150,34 +20351,34 @@
         <v>0</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>514</v>
+        <v>525</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>515</v>
+        <v>526</v>
       </c>
       <c r="D1" s="22" t="s">
-        <v>516</v>
+        <v>527</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>518</v>
+        <v>529</v>
       </c>
       <c r="G1" s="23" t="s">
-        <v>519</v>
+        <v>530</v>
       </c>
       <c r="H1" s="23" t="s">
-        <v>520</v>
+        <v>531</v>
       </c>
       <c r="I1" s="23" t="s">
-        <v>521</v>
+        <v>532</v>
       </c>
       <c r="J1" s="23" t="s">
-        <v>522</v>
+        <v>533</v>
       </c>
       <c r="K1" s="23" t="s">
-        <v>523</v>
+        <v>534</v>
       </c>
     </row>
     <row r="2" ht="126" customHeight="1">
@@ -20205,10 +20406,10 @@
       <c r="H2" s="6"/>
       <c r="I2" s="6"/>
       <c r="J2" s="6" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>525</v>
+        <v>536</v>
       </c>
     </row>
     <row r="3">
@@ -20225,7 +20426,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>526</v>
+        <v>537</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>127</v>
@@ -20236,7 +20437,7 @@
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
       <c r="J3" s="6" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="K3" s="8"/>
     </row>
@@ -20254,7 +20455,7 @@
         <v>2</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>528</v>
+        <v>539</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>127</v>
@@ -20263,10 +20464,10 @@
         <v>127</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>529</v>
+        <v>540</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="J4" s="6"/>
       <c r="K4" s="8"/>
@@ -20294,10 +20495,10 @@
         <v>127</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>532</v>
+        <v>543</v>
       </c>
       <c r="J5" s="6"/>
       <c r="K5" s="8"/>
@@ -20307,7 +20508,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>533</v>
+        <v>544</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="5"/>
@@ -20345,7 +20546,7 @@
         <v>190</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="J7" s="6"/>
       <c r="K7" s="8"/>
@@ -20393,7 +20594,7 @@
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
       <c r="K9" s="11" t="s">
-        <v>534</v>
+        <v>545</v>
       </c>
     </row>
     <row r="10">
@@ -20420,7 +20621,7 @@
       </c>
       <c r="H10" s="6"/>
       <c r="I10" s="6" t="s">
-        <v>535</v>
+        <v>546</v>
       </c>
       <c r="J10" s="6"/>
       <c r="K10" s="8"/>
@@ -20439,7 +20640,7 @@
         <v>14</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>536</v>
+        <v>547</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>45</v>
@@ -20448,12 +20649,12 @@
         <v>45</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="11" t="s">
-        <v>538</v>
+        <v>549</v>
       </c>
     </row>
     <row r="12" ht="58.5" customHeight="1">
@@ -20480,13 +20681,13 @@
       </c>
       <c r="H12" s="6"/>
       <c r="I12" s="6" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
     </row>
     <row r="13">
@@ -20539,10 +20740,10 @@
         <v>127</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>529</v>
+        <v>540</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>532</v>
+        <v>543</v>
       </c>
       <c r="J14" s="6"/>
       <c r="K14" s="8"/>
@@ -20568,10 +20769,10 @@
         <v>127</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="J15" s="6"/>
       <c r="K15" s="8" t="s">
@@ -20592,7 +20793,7 @@
         <v>3</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>45</v>
@@ -20601,14 +20802,14 @@
         <v>127</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>543</v>
+        <v>554</v>
       </c>
       <c r="J16" s="6"/>
       <c r="K16" s="8" t="s">
-        <v>544</v>
+        <v>555</v>
       </c>
     </row>
     <row r="17" ht="134" customHeight="1">
@@ -20634,16 +20835,16 @@
         <v>45</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>545</v>
+        <v>556</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>546</v>
+        <v>557</v>
       </c>
     </row>
     <row r="18">
@@ -20651,7 +20852,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>547</v>
+        <v>558</v>
       </c>
       <c r="C18" s="14" t="s">
         <v>50</v>
@@ -20660,7 +20861,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>548</v>
+        <v>559</v>
       </c>
       <c r="F18" s="14" t="s">
         <v>127</v>
@@ -20669,10 +20870,10 @@
         <v>127</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>529</v>
+        <v>540</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="J18" s="13"/>
       <c r="K18" s="15"/>
@@ -20682,7 +20883,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>549</v>
+        <v>560</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>50</v>
@@ -20691,7 +20892,7 @@
         <v>2</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>550</v>
+        <v>561</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>127</v>
@@ -20709,7 +20910,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>551</v>
+        <v>562</v>
       </c>
       <c r="C20" s="18" t="s">
         <v>50</v>
@@ -20736,7 +20937,7 @@
         <v>21</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>552</v>
+        <v>563</v>
       </c>
       <c r="C21" s="18" t="s">
         <v>50</v>
@@ -20781,10 +20982,10 @@
         <v>127</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>553</v>
+        <v>564</v>
       </c>
       <c r="J22" s="6"/>
       <c r="K22" s="6" t="s">
@@ -20828,7 +21029,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>554</v>
+        <v>565</v>
       </c>
       <c r="F24" s="21" t="s">
         <v>127</v>
@@ -20840,7 +21041,7 @@
       <c r="I24" s="17"/>
       <c r="J24" s="17"/>
       <c r="K24" s="8" t="s">
-        <v>555</v>
+        <v>566</v>
       </c>
     </row>
     <row r="25">
@@ -20848,7 +21049,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>556</v>
+        <v>567</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>50</v>
@@ -20875,7 +21076,7 @@
         <v>27</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>557</v>
+        <v>568</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>50</v>
@@ -20911,7 +21112,7 @@
         <v>2</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>558</v>
+        <v>569</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>127</v>
@@ -20931,7 +21132,7 @@
         <v>29</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>559</v>
+        <v>570</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>50</v>
@@ -20952,7 +21153,7 @@
       <c r="I28" s="6"/>
       <c r="J28" s="6"/>
       <c r="K28" s="8" t="s">
-        <v>560</v>
+        <v>571</v>
       </c>
     </row>
     <row r="29" ht="68.5" customHeight="1">
@@ -20960,7 +21161,7 @@
         <v>30</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>561</v>
+        <v>572</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>50</v>
@@ -20981,7 +21182,7 @@
       <c r="I29" s="6"/>
       <c r="J29" s="6"/>
       <c r="K29" s="8" t="s">
-        <v>562</v>
+        <v>573</v>
       </c>
     </row>
   </sheetData>
@@ -21016,7 +21217,7 @@
       <c r="A1" s="24"/>
       <c r="B1" s="24"/>
       <c r="C1" s="315" t="s">
-        <v>563</v>
+        <v>574</v>
       </c>
       <c r="D1" s="316"/>
       <c r="E1" s="316"/>
@@ -21027,7 +21228,7 @@
       <c r="J1" s="316"/>
       <c r="K1" s="317"/>
       <c r="L1" s="318" t="s">
-        <v>564</v>
+        <v>575</v>
       </c>
       <c r="M1" s="319"/>
       <c r="N1" s="319"/>
@@ -21037,7 +21238,7 @@
       <c r="B2" s="24"/>
       <c r="C2" s="25"/>
       <c r="D2" s="320" t="s">
-        <v>565</v>
+        <v>576</v>
       </c>
       <c r="E2" s="320"/>
       <c r="F2" s="320"/>
@@ -21045,7 +21246,7 @@
       <c r="H2" s="320"/>
       <c r="I2" s="320"/>
       <c r="J2" s="26" t="s">
-        <v>566</v>
+        <v>577</v>
       </c>
       <c r="K2" s="27"/>
       <c r="L2" s="25"/>
@@ -21054,66 +21255,66 @@
     </row>
     <row r="3" ht="43.5">
       <c r="A3" s="28" t="s">
-        <v>567</v>
+        <v>578</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>568</v>
+        <v>579</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>569</v>
+        <v>580</v>
       </c>
       <c r="D3" s="29" t="s">
-        <v>570</v>
+        <v>581</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>571</v>
+        <v>582</v>
       </c>
       <c r="F3" s="29" t="s">
-        <v>572</v>
+        <v>583</v>
       </c>
       <c r="G3" s="29" t="s">
-        <v>573</v>
+        <v>584</v>
       </c>
       <c r="H3" s="29" t="s">
-        <v>574</v>
+        <v>585</v>
       </c>
       <c r="I3" s="29" t="s">
-        <v>575</v>
+        <v>586</v>
       </c>
       <c r="J3" s="29" t="s">
-        <v>576</v>
+        <v>587</v>
       </c>
       <c r="K3" s="30" t="s">
-        <v>577</v>
+        <v>588</v>
       </c>
       <c r="L3" s="29" t="s">
-        <v>578</v>
+        <v>589</v>
       </c>
       <c r="M3" s="29" t="s">
-        <v>579</v>
+        <v>590</v>
       </c>
       <c r="N3" s="29" t="s">
-        <v>580</v>
+        <v>591</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="24" t="s">
-        <v>581</v>
+        <v>592</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>582</v>
+        <v>593</v>
       </c>
       <c r="C4" s="25" t="s">
         <v>127</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="E4" s="32" t="s">
         <v>63</v>
       </c>
       <c r="F4" s="32" t="s">
-        <v>584</v>
+        <v>595</v>
       </c>
       <c r="G4" s="25">
         <v>0</v>
@@ -21122,7 +21323,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="32" t="s">
-        <v>584</v>
+        <v>595</v>
       </c>
       <c r="J4" s="33" t="s">
         <v>63</v>
@@ -21134,7 +21335,7 @@
         <v>45</v>
       </c>
       <c r="M4" s="25" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="N4" s="25">
         <v>10</v>
@@ -21142,16 +21343,16 @@
     </row>
     <row r="5">
       <c r="A5" s="35" t="s">
-        <v>581</v>
+        <v>592</v>
       </c>
       <c r="B5" s="36" t="s">
-        <v>585</v>
+        <v>596</v>
       </c>
       <c r="C5" s="37" t="s">
         <v>45</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="E5" s="38" t="s">
         <v>63</v>
@@ -21176,7 +21377,7 @@
         <v>45</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="N5" s="37">
         <v>4</v>
@@ -21184,7 +21385,7 @@
     </row>
     <row r="6">
       <c r="A6" s="35" t="s">
-        <v>581</v>
+        <v>592</v>
       </c>
       <c r="B6" s="36" t="s">
         <v>269</v>
@@ -21228,43 +21429,43 @@
     </row>
     <row r="7">
       <c r="A7" s="35" t="s">
-        <v>581</v>
+        <v>592</v>
       </c>
       <c r="B7" s="36" t="s">
-        <v>587</v>
+        <v>598</v>
       </c>
       <c r="C7" s="37" t="s">
         <v>45</v>
       </c>
       <c r="D7" s="37" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="F7" s="37" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="G7" s="37" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="H7" s="37" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="I7" s="37" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="J7" s="39" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="K7" s="39" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="L7" s="37" t="s">
         <v>45</v>
       </c>
       <c r="M7" s="37" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="N7" s="37">
         <v>6</v>
@@ -21272,16 +21473,16 @@
     </row>
     <row r="8">
       <c r="A8" s="35" t="s">
-        <v>581</v>
+        <v>592</v>
       </c>
       <c r="B8" s="36" t="s">
-        <v>588</v>
+        <v>599</v>
       </c>
       <c r="C8" s="37" t="s">
         <v>45</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="E8" s="41">
         <v>0.5</v>
@@ -21300,13 +21501,13 @@
         <v>48</v>
       </c>
       <c r="K8" s="40" t="s">
-        <v>589</v>
+        <v>600</v>
       </c>
       <c r="L8" s="37" t="s">
         <v>45</v>
       </c>
       <c r="M8" s="25" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="N8" s="37">
         <v>8</v>
@@ -21317,13 +21518,13 @@
         <v>59</v>
       </c>
       <c r="B9" s="42" t="s">
-        <v>590</v>
+        <v>601</v>
       </c>
       <c r="C9" s="43" t="s">
         <v>45</v>
       </c>
       <c r="D9" s="43" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="E9" s="41" t="s">
         <v>63</v>
@@ -21350,7 +21551,7 @@
         <v>45</v>
       </c>
       <c r="M9" s="43" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="N9" s="43">
         <v>1</v>
@@ -21367,7 +21568,7 @@
         <v>45</v>
       </c>
       <c r="D10" s="47" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="E10" s="41">
         <v>1</v>
@@ -21385,16 +21586,16 @@
         <v>63</v>
       </c>
       <c r="J10" s="44" t="s">
-        <v>591</v>
+        <v>602</v>
       </c>
       <c r="K10" s="45" t="s">
-        <v>592</v>
+        <v>603</v>
       </c>
       <c r="L10" s="43" t="s">
         <v>45</v>
       </c>
       <c r="M10" s="47" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="N10" s="43">
         <v>3</v>
@@ -21405,13 +21606,13 @@
         <v>59</v>
       </c>
       <c r="B11" s="46" t="s">
-        <v>593</v>
+        <v>604</v>
       </c>
       <c r="C11" s="43" t="s">
         <v>45</v>
       </c>
       <c r="D11" s="47" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="E11" s="41">
         <v>1</v>
@@ -21429,16 +21630,16 @@
         <v>63</v>
       </c>
       <c r="J11" s="44" t="s">
-        <v>591</v>
+        <v>602</v>
       </c>
       <c r="K11" s="45" t="s">
-        <v>592</v>
+        <v>603</v>
       </c>
       <c r="L11" s="43" t="s">
         <v>45</v>
       </c>
       <c r="M11" s="47" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="N11" s="43">
         <v>3</v>
@@ -21455,7 +21656,7 @@
         <v>45</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="E12" s="49">
         <v>0.8</v>
@@ -21476,13 +21677,13 @@
         <v>253</v>
       </c>
       <c r="K12" s="52" t="s">
+        <v>605</v>
+      </c>
+      <c r="L12" s="43" t="s">
+        <v>45</v>
+      </c>
+      <c r="M12" s="43" t="s">
         <v>594</v>
-      </c>
-      <c r="L12" s="43" t="s">
-        <v>45</v>
-      </c>
-      <c r="M12" s="43" t="s">
-        <v>583</v>
       </c>
       <c r="N12" s="43">
         <v>12</v>
@@ -21493,13 +21694,13 @@
         <v>59</v>
       </c>
       <c r="B13" s="42" t="s">
-        <v>595</v>
+        <v>606</v>
       </c>
       <c r="C13" s="43" t="s">
         <v>45</v>
       </c>
       <c r="D13" s="43" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="E13" s="41">
         <v>0.5</v>
@@ -21517,7 +21718,7 @@
         <v>63</v>
       </c>
       <c r="J13" s="51" t="s">
-        <v>596</v>
+        <v>607</v>
       </c>
       <c r="K13" s="54">
         <v>9618241586</v>
@@ -21526,7 +21727,7 @@
         <v>45</v>
       </c>
       <c r="M13" s="43" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="N13" s="43">
         <v>0</v>
@@ -21537,7 +21738,7 @@
         <v>59</v>
       </c>
       <c r="B14" s="55" t="s">
-        <v>597</v>
+        <v>608</v>
       </c>
       <c r="C14" s="43" t="s">
         <v>127</v>
@@ -21614,7 +21815,7 @@
         <v>45</v>
       </c>
       <c r="M15" s="43" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="N15" s="43">
         <v>3</v>
@@ -21646,13 +21847,13 @@
         <v>210</v>
       </c>
       <c r="I16" s="43" t="s">
-        <v>598</v>
+        <v>609</v>
       </c>
       <c r="J16" s="44" t="s">
-        <v>599</v>
+        <v>610</v>
       </c>
       <c r="K16" s="45" t="s">
-        <v>600</v>
+        <v>611</v>
       </c>
       <c r="L16" s="43" t="s">
         <v>127</v>
@@ -21669,13 +21870,13 @@
         <v>59</v>
       </c>
       <c r="B17" s="46" t="s">
-        <v>601</v>
+        <v>612</v>
       </c>
       <c r="C17" s="43" t="s">
         <v>45</v>
       </c>
       <c r="D17" s="43" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="E17" s="41" t="s">
         <v>63</v>
@@ -21713,13 +21914,13 @@
         <v>59</v>
       </c>
       <c r="B18" s="46" t="s">
-        <v>602</v>
+        <v>613</v>
       </c>
       <c r="C18" s="43" t="s">
         <v>45</v>
       </c>
       <c r="D18" s="43" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="E18" s="41">
         <v>0.5</v>
@@ -21737,16 +21938,16 @@
         <v>46049</v>
       </c>
       <c r="J18" s="44" t="s">
-        <v>603</v>
+        <v>614</v>
       </c>
       <c r="K18" s="45" t="s">
-        <v>604</v>
+        <v>615</v>
       </c>
       <c r="L18" s="43" t="s">
         <v>45</v>
       </c>
       <c r="M18" s="43" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="N18" s="43">
         <v>9</v>
@@ -21763,22 +21964,22 @@
         <v>45</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>605</v>
+        <v>616</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>513</v>
+        <v>521</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>606</v>
+        <v>617</v>
       </c>
       <c r="J19" s="0" t="s">
-        <v>607</v>
+        <v>618</v>
       </c>
       <c r="K19" s="0" t="s">
-        <v>608</v>
+        <v>619</v>
       </c>
     </row>
   </sheetData>
@@ -21805,19 +22006,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="76" t="s">
-        <v>609</v>
+        <v>620</v>
       </c>
       <c r="B1" s="76" t="s">
-        <v>610</v>
+        <v>621</v>
       </c>
       <c r="C1" s="76" t="s">
-        <v>611</v>
+        <v>622</v>
       </c>
       <c r="D1" s="76" t="s">
-        <v>612</v>
+        <v>623</v>
       </c>
       <c r="E1" s="76" t="s">
-        <v>613</v>
+        <v>624</v>
       </c>
     </row>
     <row r="2">
@@ -21826,7 +22027,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>614</v>
+        <v>625</v>
       </c>
       <c r="C2" s="65" t="e">
         <f>COUNTIFS([1]Team!L1:L679, "Y", [1]Team!U1:U679, "Y")</f>
@@ -21844,7 +22045,7 @@
     <row r="3">
       <c r="A3" s="321"/>
       <c r="B3" s="6" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="C3" s="65" t="e">
         <f>COUNTIFS([1]Team!L1:L679, "Y", [1]Team!V1:V679, "Y")</f>
@@ -21862,7 +22063,7 @@
     <row r="4">
       <c r="A4" s="321"/>
       <c r="B4" s="6" t="s">
-        <v>512</v>
+        <v>520</v>
       </c>
       <c r="C4" s="65" t="e">
         <f>COUNTIFS([1]Team!L1:L679, "Y", [1]Team!AB1:AB679, "Y")</f>
@@ -21879,20 +22080,20 @@
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>615</v>
+        <v>626</v>
       </c>
       <c r="B6" s="66"/>
       <c r="C6" s="67" t="s">
-        <v>611</v>
+        <v>622</v>
       </c>
       <c r="D6" s="67" t="s">
-        <v>612</v>
+        <v>623</v>
       </c>
       <c r="E6" s="6"/>
     </row>
     <row r="7">
       <c r="B7" s="6" t="s">
-        <v>616</v>
+        <v>627</v>
       </c>
       <c r="C7" s="68">
         <v>36</v>
@@ -21904,12 +22105,12 @@
     </row>
     <row r="9">
       <c r="A9" s="322" t="s">
-        <v>617</v>
+        <v>628</v>
       </c>
       <c r="B9" s="322"/>
       <c r="C9" s="322"/>
       <c r="D9" s="0" t="s">
-        <v>618</v>
+        <v>629</v>
       </c>
     </row>
     <row r="10">
@@ -21918,12 +22119,12 @@
         <v>36</v>
       </c>
       <c r="C10" s="69" t="s">
-        <v>619</v>
+        <v>630</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="70" t="s">
-        <v>620</v>
+        <v>631</v>
       </c>
       <c r="B11" s="323">
         <v>74</v>
@@ -21932,7 +22133,7 @@
     </row>
     <row r="12">
       <c r="A12" s="71" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="B12" s="72">
         <v>61</v>
@@ -21943,7 +22144,7 @@
     </row>
     <row r="13">
       <c r="A13" s="71" t="s">
-        <v>622</v>
+        <v>633</v>
       </c>
       <c r="B13" s="73" t="e">
         <f>COUNTIFS([1]Team!L1:L679, "Y")</f>
@@ -21955,7 +22156,7 @@
     </row>
     <row r="14">
       <c r="A14" s="71" t="s">
-        <v>623</v>
+        <v>634</v>
       </c>
       <c r="B14" s="73" t="e">
         <f>COUNTIFS([1]Team!L1:L679, "N")</f>
@@ -21965,7 +22166,7 @@
     </row>
     <row r="15">
       <c r="A15" s="74" t="s">
-        <v>624</v>
+        <v>635</v>
       </c>
       <c r="B15" s="75">
         <v>26</v>
@@ -21976,14 +22177,14 @@
     </row>
     <row r="16">
       <c r="A16" s="71" t="s">
-        <v>625</v>
+        <v>636</v>
       </c>
       <c r="B16" s="72">
         <f>B12-B15</f>
         <v>35</v>
       </c>
       <c r="C16" s="71" t="s">
-        <v>626</v>
+        <v>637</v>
       </c>
     </row>
   </sheetData>

</xml_diff>